<commit_message>
Kaan teklif şablonuna Kaan Kablo Market ve Kaan Elektrik logoları eklendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EQEYJfDuBv3YycCTqCV84T
</commit_message>
<xml_diff>
--- a/alker-teklif/Kaan_Elektrik_Fiyat_Teklifi.xlsx
+++ b/alker-teklif/Kaan_Elektrik_Fiyat_Teklifi.xlsx
@@ -57,17 +57,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
-  <si>
-    <t xml:space="preserve">KAAN ELEKTRİK</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t xml:space="preserve">FİYAT TEKLİFİ</t>
   </si>
   <si>
-    <t xml:space="preserve">Otomasyon Sistemleri</t>
-  </si>
-  <si>
     <t xml:space="preserve">MÜŞTERİ</t>
   </si>
   <si>
@@ -158,7 +152,7 @@
     <t xml:space="preserve">Ödeme koşulları: %50 başlangıçta, %50 teslimde.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kaan Elektrik</t>
+    <t xml:space="preserve">Kaan Kablo Market · Kaan Elektrik</t>
   </si>
   <si>
     <t xml:space="preserve">Kaşe / İmza</t>
@@ -175,7 +169,7 @@
     <numFmt numFmtId="167" formatCode="#,##0.00&quot; ₺&quot;;\-#,##0.00&quot; ₺&quot;;\-"/>
     <numFmt numFmtId="168" formatCode="0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,23 +194,8 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="18"/>
-      <color rgb="FF0043DA"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="14"/>
       <color rgb="FF141515"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF60646A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -240,6 +219,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF141515"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF60646A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -367,32 +353,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -400,95 +390,83 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -571,13 +549,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>38160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>380520</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>624240</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>304560</xdr:rowOff>
+      <xdr:rowOff>875880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -590,8 +568,45 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="380520" cy="304560"/>
+          <a:off x="0" y="38160"/>
+          <a:ext cx="1047240" cy="837720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>781200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>38160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1695240</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>875880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1204200" y="38160"/>
+          <a:ext cx="914040" cy="837720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -798,436 +813,429 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="62"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+    <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="3" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="6" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="E7" s="7" t="n">
+        <v>46315</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="9" t="n">
-        <v>46315</v>
-      </c>
-      <c r="G7" s="10" t="s">
+      <c r="E8" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5" t="s">
+      <c r="G8" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="6" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="E9" s="9" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="11" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="10" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G10" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="C11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="D11" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="E11" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="G11" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="n">
+      <c r="A12" s="13" t="n">
         <f aca="false">IF(B12="","",ROW()-11)</f>
         <v>1</v>
       </c>
-      <c r="B12" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="17" t="n">
+      <c r="B12" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="16" t="n">
         <v>1250</v>
       </c>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="17" t="n">
         <f aca="false">IF(OR(C12="",D12=""),"",C12*D12)</f>
         <v>2500</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="str">
+        <f aca="false">IF(B13="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="21" t="str">
+        <f aca="false">IF(OR(C13="",D13=""),"",C13*D13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="str">
+        <f aca="false">IF(B14="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B14" s="14"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="17" t="str">
+        <f aca="false">IF(OR(C14="",D14=""),"",C14*D14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="str">
-        <f aca="false">IF(B13="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23" t="str">
-        <f aca="false">IF(OR(C13="",D13=""),"",C13*D13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="10" t="s">
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="str">
+        <f aca="false">IF(B15="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="21" t="str">
+        <f aca="false">IF(OR(C15="",D15=""),"",C15*D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="str">
+        <f aca="false">IF(B16="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="17" t="str">
+        <f aca="false">IF(OR(C16="",D16=""),"",C16*D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="str">
+        <f aca="false">IF(B17="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="21" t="str">
+        <f aca="false">IF(OR(C17="",D17=""),"",C17*D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="str">
+        <f aca="false">IF(B18="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B18" s="14"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17" t="str">
+        <f aca="false">IF(OR(C18="",D18=""),"",C18*D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="str">
+        <f aca="false">IF(B19="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="21" t="str">
+        <f aca="false">IF(OR(C19="",D19=""),"",C19*D19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="str">
+        <f aca="false">IF(B20="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B20" s="14"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="17" t="str">
+        <f aca="false">IF(OR(C20="",D20=""),"",C20*D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="str">
+        <f aca="false">IF(B21="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B21" s="19"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="21" t="str">
+        <f aca="false">IF(OR(C21="",D21=""),"",C21*D21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="str">
+        <f aca="false">IF(B22="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B22" s="14"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="17" t="str">
+        <f aca="false">IF(OR(C22="",D22=""),"",C22*D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="str">
+        <f aca="false">IF(B23="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="21" t="str">
+        <f aca="false">IF(OR(C23="",D23=""),"",C23*D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="str">
+        <f aca="false">IF(B24="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B24" s="14"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="17" t="str">
+        <f aca="false">IF(OR(C24="",D24=""),"",C24*D24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="str">
+        <f aca="false">IF(B25="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="21" t="str">
+        <f aca="false">IF(OR(C25="",D25=""),"",C25*D25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="str">
+        <f aca="false">IF(B26="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B26" s="14"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="17" t="str">
+        <f aca="false">IF(OR(C26="",D26=""),"",C26*D26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="str">
+        <f aca="false">IF(B27="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="21" t="str">
+        <f aca="false">IF(OR(C27="",D27=""),"",C27*D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="str">
+        <f aca="false">IF(B28="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B28" s="14"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="17" t="str">
+        <f aca="false">IF(OR(C28="",D28=""),"",C28*D28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="str">
+        <f aca="false">IF(B29="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B29" s="19"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="21" t="str">
+        <f aca="false">IF(OR(C29="",D29=""),"",C29*D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="13" t="str">
+        <f aca="false">IF(B30="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B30" s="14"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="17" t="str">
+        <f aca="false">IF(OR(C30="",D30=""),"",C30*D30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="str">
+        <f aca="false">IF(B31="","",ROW()-11)</f>
+        <v/>
+      </c>
+      <c r="B31" s="19"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="20"/>
+      <c r="E31" s="21" t="str">
+        <f aca="false">IF(OR(C31="",D31=""),"",C31*D31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D33" s="22" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="str">
-        <f aca="false">IF(B14="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="19" t="str">
-        <f aca="false">IF(OR(C14="",D14=""),"",C14*D14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="str">
-        <f aca="false">IF(B15="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23" t="str">
-        <f aca="false">IF(OR(C15="",D15=""),"",C15*D15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="str">
-        <f aca="false">IF(B16="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="19" t="str">
-        <f aca="false">IF(OR(C16="",D16=""),"",C16*D16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20" t="str">
-        <f aca="false">IF(B17="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23" t="str">
-        <f aca="false">IF(OR(C17="",D17=""),"",C17*D17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="str">
-        <f aca="false">IF(B18="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="19" t="str">
-        <f aca="false">IF(OR(C18="",D18=""),"",C18*D18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20" t="str">
-        <f aca="false">IF(B19="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="23" t="str">
-        <f aca="false">IF(OR(C19="",D19=""),"",C19*D19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="str">
-        <f aca="false">IF(B20="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="19" t="str">
-        <f aca="false">IF(OR(C20="",D20=""),"",C20*D20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="str">
-        <f aca="false">IF(B21="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="23" t="str">
-        <f aca="false">IF(OR(C21="",D21=""),"",C21*D21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="str">
-        <f aca="false">IF(B22="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B22" s="16"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="19" t="str">
-        <f aca="false">IF(OR(C22="",D22=""),"",C22*D22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="str">
-        <f aca="false">IF(B23="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="23" t="str">
-        <f aca="false">IF(OR(C23="",D23=""),"",C23*D23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="str">
-        <f aca="false">IF(B24="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="19" t="str">
-        <f aca="false">IF(OR(C24="",D24=""),"",C24*D24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="str">
-        <f aca="false">IF(B25="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B25" s="21"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="23" t="str">
-        <f aca="false">IF(OR(C25="",D25=""),"",C25*D25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="str">
-        <f aca="false">IF(B26="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="19" t="str">
-        <f aca="false">IF(OR(C26="",D26=""),"",C26*D26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="str">
-        <f aca="false">IF(B27="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B27" s="21"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="23" t="str">
-        <f aca="false">IF(OR(C27="",D27=""),"",C27*D27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="str">
-        <f aca="false">IF(B28="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="19" t="str">
-        <f aca="false">IF(OR(C28="",D28=""),"",C28*D28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="str">
-        <f aca="false">IF(B29="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="23" t="str">
-        <f aca="false">IF(OR(C29="",D29=""),"",C29*D29)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="str">
-        <f aca="false">IF(B30="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B30" s="16"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="19" t="str">
-        <f aca="false">IF(OR(C30="",D30=""),"",C30*D30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="str">
-        <f aca="false">IF(B31="","",ROW()-11)</f>
-        <v/>
-      </c>
-      <c r="B31" s="21"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="23" t="str">
-        <f aca="false">IF(OR(C31="",D31=""),"",C31*D31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D33" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="E33" s="25" t="n">
+      <c r="E33" s="23" t="n">
         <f aca="false">SUM(E12:E31)</f>
         <v>2500</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D34" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="E34" s="26" t="n">
+      <c r="D34" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E34" s="24" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D35" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="E35" s="25" t="n">
+      <c r="D35" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" s="23" t="n">
         <f aca="false">E33*E34</f>
         <v>500</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36" s="27"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="28" t="n">
+      <c r="B36" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="26" t="n">
         <f aca="false">E33+E35</f>
         <v>3000</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="10" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="10" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E43" s="27" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="10" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E44" s="28" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E43" s="29" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E44" s="30" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>